<commit_message>
Add weightless tent feature
</commit_message>
<xml_diff>
--- a/package/translations.xlsx
+++ b/package/translations.xlsx
@@ -311,7 +311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28.42" customWidth="1" style="6" min="1" max="1"/>
@@ -456,592 +456,636 @@
     <row r="7" ht="12.8" customHeight="1" s="8">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>toggle02</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Enable Storage Chest</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>収納箱を有効化</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>启用储物箱功能</t>
+          <t>toggle10</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Enable Weightless Tents</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>テント無重量を有効化</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>启用帐篷无重量</t>
         </is>
       </c>
     </row>
     <row r="8" ht="12.8" customHeight="1" s="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>tooltip02</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Enable or disable using storage chests inside tents.</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>テント内で収納箱を使用する機能を有効または無効にします。</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>启用或禁用在帐篷内使用储物箱。</t>
+          <t>tooltip14</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Enable or disable making carried tent items weightless.</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>テントアイテムを無重量にする機能を有効または無効にします。</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>启用或禁用让携带的帐篷物品变为无重量。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="12.8" customHeight="1" s="8">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>toggle03</t>
+          <t>toggle02</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Enable Delivery Box</t>
+          <t>Enable Storage Chest</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>宅配ボックスを有効化</t>
+          <t>収納箱を有効化</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>启用宅配箱功能</t>
+          <t>启用储物箱功能</t>
         </is>
       </c>
     </row>
     <row r="10" ht="12.8" customHeight="1" s="8">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>tooltip03</t>
+          <t>tooltip02</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Enable or disable delivery box functionality inside tents.</t>
+          <t>Enable or disable using storage chests inside tents.</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>テント内で宅配ボックスを機能させるかどうかを有効または無効にします。</t>
+          <t>テント内で収納箱を使用する機能を有効または無効にします。</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>启用或禁用帐篷内的宅配箱功能。</t>
+          <t>启用或禁用在帐篷内使用储物箱。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="12.8" customHeight="1" s="8">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>toggle04</t>
+          <t>toggle03</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Enable Shipping Chest</t>
+          <t>Enable Delivery Box</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>出荷箱を有効化</t>
+          <t>宅配ボックスを有効化</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>启用出货箱功能</t>
+          <t>启用宅配箱功能</t>
         </is>
       </c>
     </row>
     <row r="12" ht="12.8" customHeight="1" s="8">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>tooltip04</t>
+          <t>tooltip03</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Enable or disable using shipping chests inside tents.</t>
+          <t>Enable or disable delivery box functionality inside tents.</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>テント内で出荷箱を使用する機能を有効または無効にします。</t>
+          <t>テント内で宅配ボックスを機能させるかどうかを有効または無効にします。</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>启用或禁用在帐篷内使用出货箱。</t>
+          <t>启用或禁用帐篷内的宅配箱功能。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="12.8" customHeight="1" s="8">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>title02</t>
+          <t>toggle04</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Fertility (choose 1)</t>
+          <t>Enable Shipping Chest</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>肥沃度（1つ選択）</t>
+          <t>出荷箱を有効化</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>肥沃度（选择 1 个）</t>
+          <t>启用出货箱功能</t>
         </is>
       </c>
     </row>
     <row r="14" ht="12.8" customHeight="1" s="8">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>toggle05</t>
+          <t>tooltip04</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Enable Max Fertility</t>
+          <t>Enable or disable using shipping chests inside tents.</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>最大肥沃度を有効化</t>
+          <t>テント内で出荷箱を使用する機能を有効または無効にします。</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>启用最大肥沃度</t>
+          <t>启用或禁用在帐篷内使用出货箱。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="12.8" customHeight="1" s="8">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>tooltip05</t>
+          <t>title02</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Enable or disable max fertility inside tents (99999).</t>
+          <t>Fertility (choose 1)</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>テント内の最大肥沃度（99999）を有効または無効にします。</t>
+          <t>肥沃度（1つ選択）</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>启用或禁用帐篷内的最大肥沃度（99999）。</t>
+          <t>肥沃度（选择 1 个）</t>
         </is>
       </c>
     </row>
     <row r="16" ht="12.8" customHeight="1" s="8">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>toggle06</t>
+          <t>toggle05</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Enable No Soil Upgrade Limit</t>
+          <t>Enable Max Fertility</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>土壌アップグレード制限を解除</t>
+          <t>最大肥沃度を有効化</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>取消土壤升级限制</t>
+          <t>启用最大肥沃度</t>
         </is>
       </c>
     </row>
     <row r="17" ht="12.8" customHeight="1" s="8">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>tooltip06</t>
+          <t>tooltip05</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Enable or disable removing the soil upgrade limit inside tents.</t>
+          <t>Enable or disable max fertility inside tents (99999).</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>テント内での土壌アップグレード制限の解除を有効または無効にします。</t>
+          <t>テント内の最大肥沃度（99999）を有効または無効にします。</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>启用或禁用移除帐篷内土壤升级限制。</t>
+          <t>启用或禁用帐篷内的最大肥沃度（99999）。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="12.8" customHeight="1" s="8">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>toggle07</t>
+          <t>toggle06</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Enable Max Electricity</t>
+          <t>Enable No Soil Upgrade Limit</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>最大電力を有効化</t>
+          <t>土壌アップグレード制限を解除</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>启用最大电力</t>
+          <t>取消土壤升级限制</t>
         </is>
       </c>
     </row>
     <row r="19" ht="12.8" customHeight="1" s="8">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>tooltip07</t>
+          <t>tooltip06</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Enable or disable max electricity inside tents (99999).</t>
+          <t>Enable or disable removing the soil upgrade limit inside tents.</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>テント内の最大電力（99999）を有効または無効にします。</t>
+          <t>テント内での土壌アップグレード制限の解除を有効または無効にします。</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>启用或禁用帐篷内的最大电力（99999）。</t>
+          <t>启用或禁用移除帐篷内土壤升级限制。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="12.8" customHeight="1" s="8">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>title03</t>
+          <t>toggle07</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Land Expansion</t>
+          <t>Enable Max Electricity</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>土地拡張</t>
+          <t>最大電力を有効化</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>土地扩张</t>
+          <t>启用最大电力</t>
         </is>
       </c>
     </row>
     <row r="21" ht="12.8" customHeight="1" s="8">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>tooltip08</t>
+          <t>tooltip07</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Expand the tent land.</t>
+          <t>Enable or disable max electricity inside tents (99999).</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>テントの敷地面積を拡張します。</t>
+          <t>テント内の最大電力（99999）を有効または無効にします。</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>扩张帐篷土地面积。</t>
+          <t>启用或禁用帐篷内的最大电力（99999）。</t>
         </is>
       </c>
     </row>
     <row r="22" ht="12.8" customHeight="1" s="8">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>title04</t>
+          <t>title03</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Zone Investment</t>
+          <t>Land Expansion</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>ゾーン投資</t>
+          <t>土地拡張</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>区域投资</t>
+          <t>土地扩张</t>
         </is>
       </c>
     </row>
     <row r="23" ht="25.35" customHeight="1" s="8">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>tooltip09</t>
+          <t>tooltip08</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Invest to raise this zone’s development and influence. Higher development improves shop inventory quality and variety.</t>
+          <t>Expand the tent land.</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>投資するとゾーンの開発度と影響力が上昇し、開発度が高いほど商店の品揃え（品質と種類）が向上します。</t>
+          <t>テントの敷地面積を拡張します。</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>投资可提升该区域的开发度与影响力；开发度越高，商店的商品品质与种类都会提升。</t>
+          <t>扩张帐篷土地面积。</t>
         </is>
       </c>
     </row>
     <row r="24" ht="12.8" customHeight="1" s="8">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>title05</t>
+          <t>title04</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Merchant Recruitment</t>
+          <t>Zone Investment</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>商人の雇用</t>
+          <t>ゾーン投資</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>商人招募</t>
+          <t>区域投资</t>
         </is>
       </c>
     </row>
     <row r="25" ht="13.4" customHeight="1" s="8">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>tooltip10</t>
+          <t>tooltip09</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Recruit a merchant. Inventory quality and variety scale with zone development.</t>
+          <t>Invest to raise this zone’s development and influence. Higher development improves shop inventory quality and variety.</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>商人を雇用します。商店の品揃え（品質と種類）はゾーン開発度に連動します。</t>
+          <t>投資するとゾーンの開発度と影響力が上昇し、開発度が高いほど商店の品揃え（品質と種類）が向上します。</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>雇佣商人。商品的品质与种类随区域开发度提升而提升。</t>
+          <t>投资可提升该区域的开发度与影响力；开发度越高，商店的商品品质与种类都会提升。</t>
         </is>
       </c>
     </row>
     <row r="26" ht="12.8" customHeight="1" s="8">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>title06</t>
+          <t>title05</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Manage Land Traits (Experimental)</t>
+          <t>Merchant Recruitment</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>土地の特徴の管理（実験的）</t>
+          <t>商人の雇用</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>管理土地特性（实验性）</t>
+          <t>商人招募</t>
         </is>
       </c>
     </row>
     <row r="27" ht="12.8" customHeight="1" s="8">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>tooltip11</t>
+          <t>tooltip10</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Change this tent’s land traits.</t>
+          <t>Recruit a merchant. Inventory quality and variety scale with zone development.</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>このテントの土地の特徴を変更します。</t>
+          <t>商人を雇用します。商店の品揃え（品質と種類）はゾーン開発度に連動します。</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>修改此帐篷的土地特性。</t>
+          <t>雇佣商人。商品的品质与种类随区域开发度提升而提升。</t>
         </is>
       </c>
     </row>
     <row r="28" ht="12.8" customHeight="1" s="8">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>toggle08</t>
+          <t>title06</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Enable Teleporter</t>
+          <t>Manage Land Traits (Experimental)</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>テレポーターを有効化</t>
+          <t>土地の特徴の管理（実験的）</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>启用传送装置</t>
+          <t>管理土地特性（实验性）</t>
         </is>
       </c>
     </row>
     <row r="29" ht="12.8" customHeight="1" s="8">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>tooltip12</t>
+          <t>tooltip11</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Enable or disable the use of teleporters inside tents.</t>
+          <t>Change this tent’s land traits.</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>テント内で「テレポーター」を使用できるかを有効または無効にします。</t>
+          <t>このテントの土地の特徴を変更します。</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>启用或禁用帐篷内使用传送装置（Teleporter）。</t>
+          <t>修改此帐篷的土地特性。</t>
         </is>
       </c>
     </row>
     <row r="30" ht="12.8" customHeight="1" s="8">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>toggle09</t>
+          <t>toggle08</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Enable Dining Spot Sign</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>食堂の立て札を有効化</t>
-        </is>
-      </c>
-      <c r="D30" s="11" t="inlineStr">
-        <is>
-          <t>启用食堂招牌</t>
+          <t>Enable Teleporter</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>テレポーターを有効化</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>启用传送装置</t>
         </is>
       </c>
     </row>
     <row r="31" ht="12.8" customHeight="1" s="8">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>tooltip13</t>
+          <t>tooltip12</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Enable or disable dining spot sign effects inside tents.</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>テント内で食堂の立て札の効果を有効または無効にします。</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>启用或禁用帐篷内的食堂招牌效果。</t>
+          <t>Enable or disable the use of teleporters inside tents.</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>テント内で「テレポーター」を使用できるかを有効または無効にします。</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>启用或禁用帐篷内使用传送装置（Teleporter）。</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>fertilityModeVanilla</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Vanilla</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>バニラ</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>原版</t>
+          <t>toggle09</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Enable Dining Spot Sign</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>食堂の立て札を有効化</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>启用食堂招牌</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
+          <t>tooltip13</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Enable or disable dining spot sign effects inside tents.</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>テント内で食堂の立て札の効果を有効または無効にします。</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>启用或禁用帐篷内的食堂招牌效果。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>fertilityModeVanilla</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Vanilla</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>バニラ</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>原版</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
           <t>fertilityModeVanillaTooltip</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Use vanilla tent fertility and wrench upgrade limits.</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>テントの肥沃度とレンチ強化制限をバニラのままにします。</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>保持帐篷肥沃度和扳手升级限制为原版行为。</t>
         </is>

</xml_diff>